<commit_message>
feat: renomear UAS -> UAF (Unidade de Administração e Finanças) em todo o sistema
</commit_message>
<xml_diff>
--- a/public/modelo-disc-aderencia.xlsx
+++ b/public/modelo-disc-aderencia.xlsx
@@ -759,10 +759,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>UAS</v>
+        <v>UAF</v>
       </c>
       <c r="B21" t="str">
-        <v>Unidade de Acesso a Serviços</v>
+        <v>Unidade de Administração e Finanças</v>
       </c>
     </row>
     <row r="22">

</xml_diff>